<commit_message>
Sales follow-ups: Jersey manager script kind, export columns, template
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/powerplay-call-list-template.xlsx
+++ b/public/templates/powerplay-call-list-template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="196">
   <si>
     <t>orgType</t>
   </si>
@@ -442,27 +442,15 @@
     <t>Discovery</t>
   </si>
   <si>
+    <t>Jersey manager</t>
+  </si>
+  <si>
+    <t>Who handles the jerseys for [Org] — is that you, or someone else?</t>
+  </si>
+  <si>
     <t>Question</t>
   </si>
   <si>
-    <t>Who looks after jerseys for [Org] — is that you, an equipment manager, or does the board decide?</t>
-  </si>
-  <si>
-    <t>This person</t>
-  </si>
-  <si>
-    <t>Equipment manager</t>
-  </si>
-  <si>
-    <t>Board vote</t>
-  </si>
-  <si>
-    <t>Coach/manager per team</t>
-  </si>
-  <si>
-    <t>Parent committee</t>
-  </si>
-  <si>
     <t>When do you usually place your jersey order — and when's the next one?</t>
   </si>
   <si>
@@ -604,7 +592,7 @@
     <t>SCRIPT TAB — one row per line of the call, top to bottom within each Section (Opening, Discovery, Objections, Close).</t>
   </si>
   <si>
-    <t>Kind = Read: text to say. Reminder: a tick box. Question: a multiple-choice prompt (fill Option 1–6; leave all blank for a free-text answer). Objection: what they say (Text) and what you say back (Response).</t>
+    <t>Kind = Read: text to say. Reminder: a tick box. Question: a multiple-choice prompt (fill Option 1–6; leave all blank for a free-text answer). Objection: what they say (Text) and what you say back (Response). Jersey manager: asks who handles the jerseys — this person, or someone else (picked from the team's other contacts, or typed in as a new contact).</t>
   </si>
   <si>
     <t>Placeholders in Text/Response: [Name] first name (or "there"), [Full Name], [Org], [City], [Rep] (the caller), [Supplier], or any Contacts column in brackets, e.g. [Rink].</t>
@@ -1749,22 +1737,22 @@
         <v>132</v>
       </c>
       <c r="E8" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="F8" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="G8" t="s">
-        <v>146</v>
+        <v>132</v>
       </c>
       <c r="H8" t="s">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="I8" t="s">
-        <v>148</v>
+        <v>132</v>
       </c>
       <c r="J8" t="s">
-        <v>59</v>
+        <v>132</v>
       </c>
       <c r="K8" t="s">
         <v>132</v>
@@ -1775,22 +1763,22 @@
         <v>141</v>
       </c>
       <c r="B9" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>132</v>
       </c>
       <c r="E9" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="F9" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="G9" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="H9" t="s">
         <v>50</v>
@@ -1810,25 +1798,25 @@
         <v>141</v>
       </c>
       <c r="B10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="E10" t="s">
+        <v>150</v>
+      </c>
+      <c r="F10" t="s">
+        <v>151</v>
+      </c>
+      <c r="G10" t="s">
+        <v>152</v>
+      </c>
+      <c r="H10" t="s">
         <v>153</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="E10" t="s">
-        <v>154</v>
-      </c>
-      <c r="F10" t="s">
-        <v>155</v>
-      </c>
-      <c r="G10" t="s">
-        <v>156</v>
-      </c>
-      <c r="H10" t="s">
-        <v>157</v>
       </c>
       <c r="I10" t="s">
         <v>132</v>
@@ -1845,28 +1833,28 @@
         <v>141</v>
       </c>
       <c r="B11" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C11" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="E11" t="s">
+        <v>155</v>
+      </c>
+      <c r="F11" t="s">
+        <v>156</v>
+      </c>
+      <c r="G11" t="s">
+        <v>157</v>
+      </c>
+      <c r="H11" t="s">
         <v>158</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="E11" t="s">
+      <c r="I11" t="s">
         <v>159</v>
-      </c>
-      <c r="F11" t="s">
-        <v>160</v>
-      </c>
-      <c r="G11" t="s">
-        <v>161</v>
-      </c>
-      <c r="H11" t="s">
-        <v>162</v>
-      </c>
-      <c r="I11" t="s">
-        <v>163</v>
       </c>
       <c r="J11" t="s">
         <v>132</v>
@@ -1880,10 +1868,10 @@
         <v>141</v>
       </c>
       <c r="B12" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>132</v>
@@ -1915,25 +1903,25 @@
         <v>141</v>
       </c>
       <c r="B13" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C13" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="E13" t="s">
+        <v>162</v>
+      </c>
+      <c r="F13" t="s">
+        <v>163</v>
+      </c>
+      <c r="G13" t="s">
+        <v>164</v>
+      </c>
+      <c r="H13" t="s">
         <v>165</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="E13" t="s">
-        <v>166</v>
-      </c>
-      <c r="F13" t="s">
-        <v>167</v>
-      </c>
-      <c r="G13" t="s">
-        <v>168</v>
-      </c>
-      <c r="H13" t="s">
-        <v>169</v>
       </c>
       <c r="I13" t="s">
         <v>42</v>
@@ -1947,16 +1935,16 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B14" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="E14" t="s">
         <v>132</v>
@@ -1982,16 +1970,16 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>166</v>
+      </c>
+      <c r="B15" t="s">
+        <v>167</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="B15" t="s">
+      <c r="D15" s="4" t="s">
         <v>171</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>175</v>
       </c>
       <c r="E15" t="s">
         <v>132</v>
@@ -2017,16 +2005,16 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B16" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="E16" t="s">
         <v>132</v>
@@ -2052,16 +2040,16 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B17" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="E17" t="s">
         <v>132</v>
@@ -2087,16 +2075,16 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B18" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="E18" t="s">
         <v>132</v>
@@ -2122,13 +2110,13 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B19" t="s">
         <v>133</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>132</v>
@@ -2157,13 +2145,13 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B20" t="s">
         <v>130</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>132</v>
@@ -2192,13 +2180,13 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B21" t="s">
         <v>130</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>132</v>
@@ -2231,7 +2219,7 @@
       <formula1>"Opening,Discovery,Objections,Close"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B2:B2000">
-      <formula1>"Read,Reminder,Question,Objection"</formula1>
+      <formula1>"Read,Reminder,Question,Objection,Jersey manager"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2249,7 +2237,7 @@
   <sheetData>
     <row r="1" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -2259,42 +2247,42 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
@@ -2304,22 +2292,22 @@
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
@@ -2329,7 +2317,7 @@
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sales: script editing rules and actions; default script trimmed to the typed discovery
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/powerplay-call-list-template.xlsx
+++ b/public/templates/powerplay-call-list-template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="176">
   <si>
     <t>orgType</t>
   </si>
@@ -451,67 +451,7 @@
     <t>Question</t>
   </si>
   <si>
-    <t>When do you usually place your jersey order — and when's the next one?</t>
-  </si>
-  <si>
-    <t>This season</t>
-  </si>
-  <si>
-    <t>Next season</t>
-  </si>
-  <si>
-    <t>No plan yet</t>
-  </si>
-  <si>
-    <t>Who are you using today, and how's that going?</t>
-  </si>
-  <si>
-    <t>Happy</t>
-  </si>
-  <si>
-    <t>Fine</t>
-  </si>
-  <si>
-    <t>Unhappy</t>
-  </si>
-  <si>
-    <t>No supplier</t>
-  </si>
-  <si>
-    <t>What's in a typical order — jerseys only, socks, pant shells? One set or home and away?</t>
-  </si>
-  <si>
-    <t>Jerseys only</t>
-  </si>
-  <si>
-    <t>Jerseys + socks</t>
-  </si>
-  <si>
-    <t>Jerseys + socks + pants</t>
-  </si>
-  <si>
-    <t>Home &amp; away sets</t>
-  </si>
-  <si>
-    <t>Association-wide</t>
-  </si>
-  <si>
     <t>Roughly how many teams and players are we talking?</t>
-  </si>
-  <si>
-    <t>When you pick a supplier, what matters most?</t>
-  </si>
-  <si>
-    <t>Turnaround</t>
-  </si>
-  <si>
-    <t>Durability</t>
-  </si>
-  <si>
-    <t>Design help</t>
-  </si>
-  <si>
-    <t>Low minimums</t>
   </si>
   <si>
     <t>Objections</t>
@@ -1470,7 +1410,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -1772,16 +1712,16 @@
         <v>132</v>
       </c>
       <c r="E9" t="s">
-        <v>146</v>
+        <v>132</v>
       </c>
       <c r="F9" t="s">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="G9" t="s">
-        <v>148</v>
+        <v>132</v>
       </c>
       <c r="H9" t="s">
-        <v>50</v>
+        <v>132</v>
       </c>
       <c r="I9" t="s">
         <v>132</v>
@@ -1795,28 +1735,28 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B10" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>132</v>
-      </c>
       <c r="E10" t="s">
-        <v>150</v>
+        <v>132</v>
       </c>
       <c r="F10" t="s">
-        <v>151</v>
+        <v>132</v>
       </c>
       <c r="G10" t="s">
-        <v>152</v>
+        <v>132</v>
       </c>
       <c r="H10" t="s">
-        <v>153</v>
+        <v>132</v>
       </c>
       <c r="I10" t="s">
         <v>132</v>
@@ -1830,31 +1770,31 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B11" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="E11" t="s">
-        <v>155</v>
+        <v>132</v>
       </c>
       <c r="F11" t="s">
-        <v>156</v>
+        <v>132</v>
       </c>
       <c r="G11" t="s">
-        <v>157</v>
+        <v>132</v>
       </c>
       <c r="H11" t="s">
-        <v>158</v>
+        <v>132</v>
       </c>
       <c r="I11" t="s">
-        <v>159</v>
+        <v>132</v>
       </c>
       <c r="J11" t="s">
         <v>132</v>
@@ -1865,16 +1805,16 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B12" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>132</v>
+        <v>153</v>
       </c>
       <c r="E12" t="s">
         <v>132</v>
@@ -1900,34 +1840,34 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B13" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>132</v>
+        <v>155</v>
       </c>
       <c r="E13" t="s">
-        <v>162</v>
+        <v>132</v>
       </c>
       <c r="F13" t="s">
-        <v>163</v>
+        <v>132</v>
       </c>
       <c r="G13" t="s">
-        <v>164</v>
+        <v>132</v>
       </c>
       <c r="H13" t="s">
-        <v>165</v>
+        <v>132</v>
       </c>
       <c r="I13" t="s">
-        <v>42</v>
+        <v>132</v>
       </c>
       <c r="J13" t="s">
-        <v>59</v>
+        <v>132</v>
       </c>
       <c r="K13" t="s">
         <v>132</v>
@@ -1935,16 +1875,16 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>166</v>
+        <v>146</v>
       </c>
       <c r="B14" t="s">
-        <v>167</v>
+        <v>147</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="E14" t="s">
         <v>132</v>
@@ -1970,16 +1910,16 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="B15" t="s">
-        <v>167</v>
+        <v>133</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>171</v>
+        <v>132</v>
       </c>
       <c r="E15" t="s">
         <v>132</v>
@@ -2005,16 +1945,16 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="B16" t="s">
-        <v>167</v>
+        <v>130</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>173</v>
+        <v>132</v>
       </c>
       <c r="E16" t="s">
         <v>132</v>
@@ -2040,16 +1980,16 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="B17" t="s">
-        <v>167</v>
+        <v>130</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>174</v>
+        <v>161</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>175</v>
+        <v>132</v>
       </c>
       <c r="E17" t="s">
         <v>132</v>
@@ -2070,146 +2010,6 @@
         <v>132</v>
       </c>
       <c r="K17" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>166</v>
-      </c>
-      <c r="B18" t="s">
-        <v>167</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="E18" t="s">
-        <v>132</v>
-      </c>
-      <c r="F18" t="s">
-        <v>132</v>
-      </c>
-      <c r="G18" t="s">
-        <v>132</v>
-      </c>
-      <c r="H18" t="s">
-        <v>132</v>
-      </c>
-      <c r="I18" t="s">
-        <v>132</v>
-      </c>
-      <c r="J18" t="s">
-        <v>132</v>
-      </c>
-      <c r="K18" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>178</v>
-      </c>
-      <c r="B19" t="s">
-        <v>133</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="E19" t="s">
-        <v>132</v>
-      </c>
-      <c r="F19" t="s">
-        <v>132</v>
-      </c>
-      <c r="G19" t="s">
-        <v>132</v>
-      </c>
-      <c r="H19" t="s">
-        <v>132</v>
-      </c>
-      <c r="I19" t="s">
-        <v>132</v>
-      </c>
-      <c r="J19" t="s">
-        <v>132</v>
-      </c>
-      <c r="K19" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>178</v>
-      </c>
-      <c r="B20" t="s">
-        <v>130</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="E20" t="s">
-        <v>132</v>
-      </c>
-      <c r="F20" t="s">
-        <v>132</v>
-      </c>
-      <c r="G20" t="s">
-        <v>132</v>
-      </c>
-      <c r="H20" t="s">
-        <v>132</v>
-      </c>
-      <c r="I20" t="s">
-        <v>132</v>
-      </c>
-      <c r="J20" t="s">
-        <v>132</v>
-      </c>
-      <c r="K20" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>178</v>
-      </c>
-      <c r="B21" t="s">
-        <v>130</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="E21" t="s">
-        <v>132</v>
-      </c>
-      <c r="F21" t="s">
-        <v>132</v>
-      </c>
-      <c r="G21" t="s">
-        <v>132</v>
-      </c>
-      <c r="H21" t="s">
-        <v>132</v>
-      </c>
-      <c r="I21" t="s">
-        <v>132</v>
-      </c>
-      <c r="J21" t="s">
-        <v>132</v>
-      </c>
-      <c r="K21" t="s">
         <v>132</v>
       </c>
     </row>
@@ -2237,7 +2037,7 @@
   <sheetData>
     <row r="1" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>182</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -2247,42 +2047,42 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>184</v>
+        <v>164</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>186</v>
+        <v>166</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>187</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>188</v>
+        <v>168</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>189</v>
+        <v>169</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>190</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
@@ -2292,22 +2092,22 @@
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>191</v>
+        <v>171</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>193</v>
+        <v>173</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>194</v>
+        <v>174</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
@@ -2317,7 +2117,7 @@
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sales call screen: exactly five discovery questions; Settings for the pickup line and voicemail; Went to voicemail
- Discovery renders only the five typed questions; the sheet's other
  discovery rows are ignored on screen and the default script drops its
  last one.
- A Settings side sheet (gear in the top bar) holds the pickup line and
  the new per-list voicemail message; the pickup line is view-only.
- Went to voicemail, in the expanded Opening, shows the message at
  read-aloud size and logs Voicemail in one click.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/powerplay-call-list-template.xlsx
+++ b/public/templates/powerplay-call-list-template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="174">
   <si>
     <t>orgType</t>
   </si>
@@ -446,12 +446,6 @@
   </si>
   <si>
     <t>Who handles the jerseys for [Org] — is that you, or someone else?</t>
-  </si>
-  <si>
-    <t>Question</t>
-  </si>
-  <si>
-    <t>Roughly how many teams and players are we talking?</t>
   </si>
   <si>
     <t>Objections</t>
@@ -1410,7 +1404,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -1700,16 +1694,16 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B9" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>132</v>
+        <v>147</v>
       </c>
       <c r="E9" t="s">
         <v>132</v>
@@ -1735,10 +1729,10 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B10" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>148</v>
@@ -1770,10 +1764,10 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B11" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>150</v>
@@ -1805,10 +1799,10 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B12" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>152</v>
@@ -1840,10 +1834,10 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B13" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>154</v>
@@ -1875,16 +1869,16 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="B14" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>157</v>
+        <v>132</v>
       </c>
       <c r="E14" t="s">
         <v>132</v>
@@ -1910,13 +1904,13 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>156</v>
+      </c>
+      <c r="B15" t="s">
+        <v>130</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>158</v>
-      </c>
-      <c r="B15" t="s">
-        <v>133</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>159</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>132</v>
@@ -1945,13 +1939,13 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B16" t="s">
         <v>130</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>132</v>
@@ -1975,41 +1969,6 @@
         <v>132</v>
       </c>
       <c r="K16" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>158</v>
-      </c>
-      <c r="B17" t="s">
-        <v>130</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="E17" t="s">
-        <v>132</v>
-      </c>
-      <c r="F17" t="s">
-        <v>132</v>
-      </c>
-      <c r="G17" t="s">
-        <v>132</v>
-      </c>
-      <c r="H17" t="s">
-        <v>132</v>
-      </c>
-      <c r="I17" t="s">
-        <v>132</v>
-      </c>
-      <c r="J17" t="s">
-        <v>132</v>
-      </c>
-      <c r="K17" t="s">
         <v>132</v>
       </c>
     </row>
@@ -2037,7 +1996,7 @@
   <sheetData>
     <row r="1" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -2047,42 +2006,42 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
@@ -2092,22 +2051,22 @@
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
@@ -2117,7 +2076,7 @@
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>